<commit_message>
synchronize local and remote
</commit_message>
<xml_diff>
--- a/Behavioral figures/Female cohort - PO/Stats - female cohort.xlsx
+++ b/Behavioral figures/Female cohort - PO/Stats - female cohort.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mchakra/Dropbox/Stanford/Research/Bhatt lab/Computation/BBB project/Paper code/Behavioral figures/Female cohort - PO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F0FD31-0A9B-B549-B5CD-D56810D140BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77F3531-648A-9A44-89E7-63D14FC9A7CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="320" yWindow="600" windowWidth="24880" windowHeight="18600" xr2:uid="{FA8177BD-2F0A-5E4A-A9D8-F2B705A8E847}"/>
+    <workbookView xWindow="22800" yWindow="2620" windowWidth="24880" windowHeight="18600" xr2:uid="{FA8177BD-2F0A-5E4A-A9D8-F2B705A8E847}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,46 +56,46 @@
     <t>Confidence interval upper bound</t>
   </si>
   <si>
-    <t>Activity chamber - total distance moved in periphery (cm) - two-sample t-test</t>
-  </si>
-  <si>
-    <t>Activity chamber - total distance moved in center (cm) - two-sample t-test</t>
-  </si>
-  <si>
-    <t>Activity chamber - total vertical counts (periphery + center) - two-sample t-test</t>
-  </si>
-  <si>
-    <t>Activity chamber - total time in center (s) - two-sample t-test</t>
-  </si>
-  <si>
-    <t>Activity chamber - latency to center (s) - two-sample t-test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y-maze - % alternation 0-5 min, vehicle group - one-sample t-test comparing to chance levels </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y-maze - % alternation 0-5 min, GDCA group - one-sample t-test comparing to chance levels </t>
-  </si>
-  <si>
-    <t>Y-maze - number of entries (0-5min) - two-sample t-test</t>
-  </si>
-  <si>
-    <t>Y-maze - total distance moved (0-5min; cm) - two-sample t-test</t>
-  </si>
-  <si>
     <t>Odds ratio</t>
   </si>
   <si>
-    <t>Rotarod - latency to fall (s) - two-sample t-test - for the 15min_32rpm condition</t>
-  </si>
-  <si>
-    <t>Rotarod - proportion of mice that fell - Fisher exact test - for the 15min_32rpm condition</t>
-  </si>
-  <si>
-    <t>% dry weight of fecal pellets - two-sample t-test</t>
-  </si>
-  <si>
-    <t>Body temperature - 60min timepoint - change vs. baseline - two-sample t-test</t>
+    <t>Activity chamber (females) - total distance moved in periphery (cm) - two-sample t-test</t>
+  </si>
+  <si>
+    <t>Activity chamber (females) - total distance moved in center (cm) - two-sample t-test</t>
+  </si>
+  <si>
+    <t>Activity chamber (females) - total vertical counts (periphery + center) - two-sample t-test</t>
+  </si>
+  <si>
+    <t>Activity chamber (females) - total time in center (s) - two-sample t-test</t>
+  </si>
+  <si>
+    <t>Activity chamber (females) - latency to center (s) - two-sample t-test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y-maze (females) - % alternation 0-5 min, vehicle group - one-sample t-test comparing to chance levels </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y-maze (females) - % alternation 0-5 min, GDCA group - one-sample t-test comparing to chance levels </t>
+  </si>
+  <si>
+    <t>Y-maze (females) - number of entries (0-5min) - two-sample t-test</t>
+  </si>
+  <si>
+    <t>Y-maze (females) - total distance moved (0-5min; cm) - two-sample t-test</t>
+  </si>
+  <si>
+    <t>Rotarod (females) - latency to fall (s) - two-sample t-test - for the 15min_32rpm condition</t>
+  </si>
+  <si>
+    <t>Rotarod (females) - proportion of mice that fell - Fisher exact test - for the 15min_32rpm condition</t>
+  </si>
+  <si>
+    <t>% dry weight of fecal pellets - females - two-sample t-test</t>
+  </si>
+  <si>
+    <t>Body temperature - females - 60min timepoint - change vs. baseline - two-sample t-test</t>
   </si>
 </sst>
 </file>
@@ -150,14 +150,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -492,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29C21E27-AE1A-BB4A-909F-F838FB776FC9}">
-  <dimension ref="A2:G63"/>
+  <dimension ref="A2:G60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
@@ -504,7 +503,7 @@
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -547,7 +546,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -590,7 +589,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -633,7 +632,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -676,7 +675,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -719,7 +718,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -762,7 +761,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -805,7 +804,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -848,7 +847,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -943,7 +942,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>2</v>
@@ -1055,30 +1054,28 @@
         <v>0.20520479999999999</v>
       </c>
     </row>
-    <row r="54" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="55" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="56" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" s="5"/>
       <c r="B56" s="5"/>
       <c r="C56" s="5"/>
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
     </row>
-    <row r="57" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" s="5"/>
       <c r="B57" s="5"/>
       <c r="C57" s="5"/>
       <c r="D57" s="5"/>
       <c r="E57" s="5"/>
     </row>
-    <row r="59" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" s="5"/>
       <c r="B59" s="5"/>
       <c r="C59" s="5"/>
       <c r="D59" s="5"/>
       <c r="E59" s="5"/>
     </row>
-    <row r="60" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" s="5"/>
       <c r="B60" s="5"/>
       <c r="C60" s="5"/>
@@ -1087,9 +1084,6 @@
       <c r="F60" s="5"/>
       <c r="G60" s="5"/>
     </row>
-    <row r="61" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="62" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="63" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>